<commit_message>
#21 BOM File Updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/BOB_MCF8316/Client_BOM_BOB.xlsx
+++ b/Deliverables/BOM/BOB_MCF8316/Client_BOM_BOB.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Mahmood-PTZKeyboard\Deliverables\BOM\BOB_MCF8316\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D82AD52A-E819-4283-B43B-5767A6B172F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434B8595-56BB-4BEE-8AAA-5A54C9952BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22305" yWindow="4815" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="175">
   <si>
     <t>Component list</t>
   </si>
@@ -446,9 +446,6 @@
     <t>Alternate Part Number</t>
   </si>
   <si>
-    <t>LCSC/Part Number</t>
-  </si>
-  <si>
     <t xml:space="preserve">Value </t>
   </si>
   <si>
@@ -488,84 +485,6 @@
     <t>IC</t>
   </si>
   <si>
-    <t>C109447</t>
-  </si>
-  <si>
-    <t>C249985</t>
-  </si>
-  <si>
-    <t>C909823</t>
-  </si>
-  <si>
-    <t>C113803</t>
-  </si>
-  <si>
-    <t>C149602</t>
-  </si>
-  <si>
-    <t>C14664</t>
-  </si>
-  <si>
-    <t>C389107</t>
-  </si>
-  <si>
-    <t>C7230</t>
-  </si>
-  <si>
-    <t>C527013</t>
-  </si>
-  <si>
-    <t>C150735</t>
-  </si>
-  <si>
-    <t>C307679</t>
-  </si>
-  <si>
-    <t>C361669</t>
-  </si>
-  <si>
-    <t>C98359</t>
-  </si>
-  <si>
-    <t>C364556</t>
-  </si>
-  <si>
-    <t>C74338</t>
-  </si>
-  <si>
-    <t>C8483</t>
-  </si>
-  <si>
-    <t>C358687</t>
-  </si>
-  <si>
-    <t>C132810</t>
-  </si>
-  <si>
-    <t>C341716</t>
-  </si>
-  <si>
-    <t>C107701</t>
-  </si>
-  <si>
-    <t>C140867</t>
-  </si>
-  <si>
-    <t>C2935237</t>
-  </si>
-  <si>
-    <t>C105428</t>
-  </si>
-  <si>
-    <t>C14677</t>
-  </si>
-  <si>
-    <t>C388633</t>
-  </si>
-  <si>
-    <t>C3003196</t>
-  </si>
-  <si>
     <t>Bill of Materials for Project [BOB]</t>
   </si>
   <si>
@@ -620,9 +539,6 @@
     <t>RC0603FR-0722RL</t>
   </si>
   <si>
-    <t>MTP125-1105S1</t>
-  </si>
-  <si>
     <t>RC0402FR-071KL</t>
   </si>
   <si>
@@ -630,6 +546,15 @@
   </si>
   <si>
     <t>Single Board Cost</t>
+  </si>
+  <si>
+    <t>MTP125-1106S1</t>
+  </si>
+  <si>
+    <t>TDK Corporation</t>
+  </si>
+  <si>
+    <t>FH</t>
   </si>
 </sst>
 </file>
@@ -1297,6 +1222,7 @@
     <xf numFmtId="166" fontId="15" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1329,7 +1255,6 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1357,13 +1282,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>17</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>10417</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>16</xdr:col>
       <xdr:colOff>1724025</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>161925</xdr:rowOff>
@@ -1671,7 +1596,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:U39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1682,19 +1607,18 @@
     <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.85546875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1704,17 +1628,16 @@
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="67"/>
-      <c r="P1" s="67"/>
-      <c r="Q1" s="67"/>
-      <c r="R1" s="68"/>
-    </row>
-    <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="68"/>
+      <c r="K1" s="68"/>
+      <c r="L1" s="68"/>
+      <c r="M1" s="68"/>
+      <c r="N1" s="68"/>
+      <c r="O1" s="68"/>
+      <c r="P1" s="68"/>
+      <c r="Q1" s="69"/>
+    </row>
+    <row r="2" spans="1:21" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="21"/>
       <c r="C2" s="39"/>
@@ -1723,7 +1646,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="55" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1735,10 +1658,9 @@
       <c r="N2" s="4"/>
       <c r="O2" s="4"/>
       <c r="P2" s="4"/>
-      <c r="Q2" s="4"/>
-      <c r="R2" s="3"/>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q2" s="3"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="22"/>
       <c r="C3" s="40"/>
@@ -1747,7 +1669,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="56" t="s">
-        <v>179</v>
+        <v>152</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1759,10 +1681,9 @@
       <c r="N3" s="5"/>
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
-      <c r="Q3" s="5"/>
-      <c r="R3" s="69"/>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q3" s="70"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="22"/>
       <c r="C4" s="40"/>
@@ -1771,22 +1692,21 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="57" t="s">
-        <v>179</v>
+        <v>152</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
       <c r="I4" s="14"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
+      <c r="K4" s="6"/>
       <c r="L4" s="6"/>
       <c r="M4" s="6"/>
       <c r="N4" s="6"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
-      <c r="Q4" s="6"/>
-      <c r="R4" s="70"/>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q4" s="71"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="22"/>
       <c r="C5" s="40"/>
@@ -1807,10 +1727,9 @@
       <c r="N5" s="6"/>
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
-      <c r="Q5" s="6"/>
-      <c r="R5" s="70"/>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q5" s="71"/>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="23"/>
       <c r="C6" s="41"/>
@@ -1827,10 +1746,9 @@
       <c r="N6" s="6"/>
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="70"/>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="Q6" s="71"/>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="24"/>
       <c r="C7" s="42"/>
@@ -1847,10 +1765,9 @@
       <c r="N7" s="8"/>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="70"/>
-    </row>
-    <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q7" s="71"/>
+    </row>
+    <row r="8" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="27"/>
       <c r="C8" s="43"/>
@@ -1867,10 +1784,9 @@
       <c r="N8" s="8"/>
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="70"/>
-    </row>
-    <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="Q8" s="71"/>
+    </row>
+    <row r="9" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="30" t="s">
         <v>4</v>
@@ -1899,39 +1815,36 @@
       <c r="J9" s="30" t="s">
         <v>138</v>
       </c>
-      <c r="K9" s="30" t="s">
+      <c r="K9" s="31" t="s">
+        <v>135</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>162</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="N9" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="P9" s="32" t="s">
         <v>139</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>135</v>
-      </c>
-      <c r="M9" s="30" t="s">
-        <v>189</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>190</v>
-      </c>
-      <c r="O9" s="30" t="s">
-        <v>191</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>192</v>
       </c>
       <c r="Q9" s="32" t="s">
         <v>140</v>
       </c>
-      <c r="R9" s="32" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="38">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D10" s="46" t="s">
         <v>7</v>
@@ -1949,44 +1862,41 @@
         <v>100</v>
       </c>
       <c r="I10" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J10" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="K10" s="46" t="s">
         <v>115</v>
       </c>
-      <c r="L10" s="47">
+      <c r="K10" s="47">
         <v>1</v>
       </c>
+      <c r="L10" s="46">
+        <f>K10*10</f>
+        <v>10</v>
+      </c>
       <c r="M10" s="46">
-        <f>L10*10</f>
-        <v>10</v>
-      </c>
-      <c r="N10" s="46">
         <v>20</v>
       </c>
+      <c r="N10" s="53">
+        <v>0.13320000000000001</v>
+      </c>
       <c r="O10" s="53">
-        <v>0.13320000000000001</v>
-      </c>
-      <c r="P10" s="53">
-        <f>O10*N10</f>
+        <f t="shared" ref="O10:O33" si="0">N10*M10</f>
         <v>2.6640000000000001</v>
       </c>
-      <c r="Q10" s="48"/>
-      <c r="R10" s="49"/>
-      <c r="T10" s="77"/>
-      <c r="V10" s="77"/>
-    </row>
-    <row r="11" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="P10" s="48"/>
+      <c r="Q10" s="49"/>
+      <c r="S10" s="67"/>
+      <c r="U10" s="67"/>
+    </row>
+    <row r="11" spans="1:21" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="38">
-        <f t="shared" ref="B11:B37" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B37" si="1">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D11" s="50" t="s">
         <v>8</v>
@@ -1995,53 +1905,50 @@
         <v>37</v>
       </c>
       <c r="F11" s="50" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="G11" s="51" t="s">
-        <v>180</v>
+        <v>153</v>
       </c>
       <c r="H11" s="50" t="s">
         <v>101</v>
       </c>
       <c r="I11" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J11" s="50" t="s">
-        <v>153</v>
-      </c>
-      <c r="K11" s="50" t="s">
         <v>116</v>
       </c>
-      <c r="L11" s="51">
+      <c r="K11" s="51">
         <v>1</v>
       </c>
+      <c r="L11" s="50">
+        <f t="shared" ref="L11:L37" si="2">K11*10</f>
+        <v>10</v>
+      </c>
       <c r="M11" s="50">
-        <f t="shared" ref="M11:M37" si="1">L11*10</f>
-        <v>10</v>
-      </c>
-      <c r="N11" s="50">
         <v>12</v>
       </c>
+      <c r="N11" s="54">
+        <v>0.47870000000000001</v>
+      </c>
       <c r="O11" s="54">
-        <v>0.47870000000000001</v>
-      </c>
-      <c r="P11" s="54">
-        <f>O11*N11</f>
+        <f t="shared" si="0"/>
         <v>5.7444000000000006</v>
       </c>
+      <c r="P11" s="52"/>
       <c r="Q11" s="52"/>
-      <c r="R11" s="52"/>
-      <c r="T11" s="77"/>
-      <c r="V11" s="77"/>
-    </row>
-    <row r="12" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S11" s="67"/>
+      <c r="U11" s="67"/>
+    </row>
+    <row r="12" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="38">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D12" s="46" t="s">
         <v>9</v>
@@ -2059,44 +1966,41 @@
         <v>102</v>
       </c>
       <c r="I12" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J12" s="46" t="s">
-        <v>154</v>
-      </c>
-      <c r="K12" s="46" t="s">
         <v>117</v>
       </c>
-      <c r="L12" s="47">
+      <c r="K12" s="47">
         <v>2</v>
       </c>
+      <c r="L12" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="M12" s="46">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N12" s="46">
         <v>25</v>
       </c>
+      <c r="N12" s="53">
+        <v>0.23780000000000001</v>
+      </c>
       <c r="O12" s="53">
-        <v>0.23780000000000001</v>
-      </c>
-      <c r="P12" s="53">
-        <f>O12*N12</f>
+        <f t="shared" si="0"/>
         <v>5.9450000000000003</v>
       </c>
+      <c r="P12" s="48"/>
       <c r="Q12" s="48"/>
-      <c r="R12" s="48"/>
-      <c r="T12" s="77"/>
-      <c r="V12" s="77"/>
-    </row>
-    <row r="13" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S12" s="67"/>
+      <c r="U12" s="67"/>
+    </row>
+    <row r="13" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C13" s="60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D13" s="50" t="s">
         <v>10</v>
@@ -2114,44 +2018,41 @@
         <v>100</v>
       </c>
       <c r="I13" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J13" s="50" t="s">
-        <v>155</v>
-      </c>
-      <c r="K13" s="50" t="s">
         <v>118</v>
       </c>
-      <c r="L13" s="51">
+      <c r="K13" s="51">
         <v>4</v>
       </c>
+      <c r="L13" s="50">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="M13" s="50">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N13" s="50">
         <v>100</v>
       </c>
+      <c r="N13" s="54">
+        <v>0.1053</v>
+      </c>
       <c r="O13" s="54">
-        <v>0.1053</v>
-      </c>
-      <c r="P13" s="54">
-        <f>O13*N13</f>
+        <f t="shared" si="0"/>
         <v>10.530000000000001</v>
       </c>
+      <c r="P13" s="52"/>
       <c r="Q13" s="52"/>
-      <c r="R13" s="52"/>
-      <c r="T13" s="77"/>
-      <c r="V13" s="77"/>
-    </row>
-    <row r="14" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S13" s="67"/>
+      <c r="U13" s="67"/>
+    </row>
+    <row r="14" spans="1:21" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="38">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D14" s="46" t="s">
         <v>11</v>
@@ -2163,48 +2064,45 @@
         <v>65</v>
       </c>
       <c r="G14" s="47" t="s">
-        <v>181</v>
+        <v>154</v>
       </c>
       <c r="H14" s="46"/>
       <c r="I14" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J14" s="46" t="s">
-        <v>156</v>
-      </c>
-      <c r="K14" s="46" t="s">
         <v>119</v>
       </c>
-      <c r="L14" s="47">
+      <c r="K14" s="47">
         <v>2</v>
       </c>
+      <c r="L14" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="M14" s="46">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N14" s="46">
         <v>50</v>
       </c>
+      <c r="N14" s="53">
+        <v>0.10840000000000001</v>
+      </c>
       <c r="O14" s="53">
-        <v>0.10840000000000001</v>
-      </c>
-      <c r="P14" s="53">
-        <f>O14*N14</f>
+        <f t="shared" si="0"/>
         <v>5.4200000000000008</v>
       </c>
+      <c r="P14" s="48"/>
       <c r="Q14" s="48"/>
-      <c r="R14" s="48"/>
-      <c r="T14" s="77"/>
-      <c r="V14" s="77"/>
-    </row>
-    <row r="15" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S14" s="67"/>
+      <c r="U14" s="67"/>
+    </row>
+    <row r="15" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C15" s="60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D15" s="50" t="s">
         <v>12</v>
@@ -2222,44 +2120,41 @@
         <v>100</v>
       </c>
       <c r="I15" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J15" s="50" t="s">
-        <v>157</v>
-      </c>
-      <c r="K15" s="50" t="s">
         <v>117</v>
       </c>
-      <c r="L15" s="51">
+      <c r="K15" s="51">
         <v>3</v>
       </c>
+      <c r="L15" s="50">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
       <c r="M15" s="50">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="N15" s="50">
         <v>100</v>
       </c>
+      <c r="N15" s="54">
+        <v>0.10600000000000001</v>
+      </c>
       <c r="O15" s="54">
-        <v>0.10600000000000001</v>
-      </c>
-      <c r="P15" s="54">
-        <f>O15*N15</f>
+        <f t="shared" si="0"/>
         <v>10.600000000000001</v>
       </c>
+      <c r="P15" s="52"/>
       <c r="Q15" s="52"/>
-      <c r="R15" s="52"/>
-      <c r="T15" s="77"/>
-      <c r="V15" s="77"/>
-    </row>
-    <row r="16" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S15" s="67"/>
+      <c r="U15" s="67"/>
+    </row>
+    <row r="16" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="38">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D16" s="46" t="s">
         <v>13</v>
@@ -2277,44 +2172,41 @@
         <v>100</v>
       </c>
       <c r="I16" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J16" s="46" t="s">
-        <v>158</v>
-      </c>
-      <c r="K16" s="46" t="s">
         <v>120</v>
       </c>
-      <c r="L16" s="47">
+      <c r="K16" s="47">
         <v>1</v>
       </c>
+      <c r="L16" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M16" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N16" s="46">
         <v>50</v>
       </c>
+      <c r="N16" s="53">
+        <v>0.11310000000000001</v>
+      </c>
       <c r="O16" s="53">
-        <v>0.11310000000000001</v>
-      </c>
-      <c r="P16" s="53">
-        <f>O16*N16</f>
+        <f t="shared" si="0"/>
         <v>5.6550000000000002</v>
       </c>
+      <c r="P16" s="48"/>
       <c r="Q16" s="48"/>
-      <c r="R16" s="48"/>
-      <c r="T16" s="77"/>
-      <c r="V16" s="77"/>
-    </row>
-    <row r="17" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S16" s="67"/>
+      <c r="U16" s="67"/>
+    </row>
+    <row r="17" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C17" s="60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D17" s="50" t="s">
         <v>14</v>
@@ -2332,44 +2224,41 @@
         <v>103</v>
       </c>
       <c r="I17" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J17" s="50" t="s">
-        <v>159</v>
-      </c>
-      <c r="K17" s="50" t="s">
         <v>121</v>
       </c>
-      <c r="L17" s="51">
+      <c r="K17" s="51">
         <v>1</v>
       </c>
+      <c r="L17" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M17" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N17" s="50">
         <v>12</v>
       </c>
+      <c r="N17" s="54">
+        <v>0.91249999999999998</v>
+      </c>
       <c r="O17" s="54">
-        <v>0.91249999999999998</v>
-      </c>
-      <c r="P17" s="54">
-        <f>O17*N17</f>
+        <f t="shared" si="0"/>
         <v>10.95</v>
       </c>
+      <c r="P17" s="52"/>
       <c r="Q17" s="52"/>
-      <c r="R17" s="52"/>
-      <c r="T17" s="77"/>
-      <c r="V17" s="77"/>
-    </row>
-    <row r="18" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S17" s="67"/>
+      <c r="U17" s="67"/>
+    </row>
+    <row r="18" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="38">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
       <c r="C18" s="59" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D18" s="46" t="s">
         <v>15</v>
@@ -2387,44 +2276,41 @@
         <v>104</v>
       </c>
       <c r="I18" s="46" t="s">
-        <v>185</v>
+        <v>158</v>
       </c>
       <c r="J18" s="46" t="s">
-        <v>160</v>
-      </c>
-      <c r="K18" s="46" t="s">
         <v>122</v>
       </c>
-      <c r="L18" s="47">
+      <c r="K18" s="47">
         <v>2</v>
       </c>
+      <c r="L18" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="M18" s="46">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N18" s="46">
         <v>100</v>
       </c>
+      <c r="N18" s="53">
+        <v>0.1046</v>
+      </c>
       <c r="O18" s="53">
-        <v>0.1046</v>
-      </c>
-      <c r="P18" s="53">
-        <f>O18*N18</f>
+        <f t="shared" si="0"/>
         <v>10.459999999999999</v>
       </c>
+      <c r="P18" s="48"/>
       <c r="Q18" s="48"/>
-      <c r="R18" s="48"/>
-      <c r="T18" s="77"/>
-      <c r="V18" s="77"/>
-    </row>
-    <row r="19" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S18" s="67"/>
+      <c r="U18" s="67"/>
+    </row>
+    <row r="19" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C19" s="60" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D19" s="50" t="s">
         <v>16</v>
@@ -2442,44 +2328,41 @@
         <v>105</v>
       </c>
       <c r="I19" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J19" s="50" t="s">
-        <v>161</v>
-      </c>
-      <c r="K19" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="L19" s="51">
+        <v>159</v>
+      </c>
+      <c r="K19" s="51">
         <v>1</v>
       </c>
+      <c r="L19" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M19" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N19" s="50">
         <v>20</v>
       </c>
+      <c r="N19" s="54">
+        <v>0.1431</v>
+      </c>
       <c r="O19" s="54">
-        <v>0.1431</v>
-      </c>
-      <c r="P19" s="54">
-        <f>O19*N19</f>
+        <f t="shared" si="0"/>
         <v>2.8620000000000001</v>
       </c>
+      <c r="P19" s="52"/>
       <c r="Q19" s="52"/>
-      <c r="R19" s="52"/>
-      <c r="T19" s="77"/>
-      <c r="V19" s="77"/>
-    </row>
-    <row r="20" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S19" s="67"/>
+      <c r="U19" s="67"/>
+    </row>
+    <row r="20" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="38">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
       <c r="C20" s="59" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D20" s="46" t="s">
         <v>17</v>
@@ -2491,48 +2374,47 @@
         <v>70</v>
       </c>
       <c r="G20" s="47" t="s">
-        <v>182</v>
-      </c>
-      <c r="H20" s="46"/>
+        <v>155</v>
+      </c>
+      <c r="H20" s="46" t="s">
+        <v>173</v>
+      </c>
       <c r="I20" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J20" s="46" t="s">
-        <v>162</v>
-      </c>
-      <c r="K20" s="46" t="s">
         <v>123</v>
       </c>
-      <c r="L20" s="47">
+      <c r="K20" s="47">
         <v>1</v>
       </c>
+      <c r="L20" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M20" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N20" s="46">
         <v>15</v>
       </c>
+      <c r="N20" s="53">
+        <v>0.2838</v>
+      </c>
       <c r="O20" s="53">
-        <v>0.2838</v>
-      </c>
-      <c r="P20" s="53">
-        <f>O20*N20</f>
+        <f t="shared" si="0"/>
         <v>4.2569999999999997</v>
       </c>
+      <c r="P20" s="48"/>
       <c r="Q20" s="48"/>
-      <c r="R20" s="48"/>
-      <c r="T20" s="77"/>
-      <c r="V20" s="77"/>
-    </row>
-    <row r="21" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S20" s="67"/>
+      <c r="U20" s="67"/>
+    </row>
+    <row r="21" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C21" s="60" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D21" s="50" t="s">
         <v>18</v>
@@ -2544,48 +2426,47 @@
         <v>70</v>
       </c>
       <c r="G21" s="51" t="s">
-        <v>183</v>
-      </c>
-      <c r="H21" s="50"/>
+        <v>156</v>
+      </c>
+      <c r="H21" s="50" t="s">
+        <v>174</v>
+      </c>
       <c r="I21" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J21" s="50" t="s">
-        <v>163</v>
-      </c>
-      <c r="K21" s="50" t="s">
         <v>124</v>
       </c>
-      <c r="L21" s="51">
+      <c r="K21" s="51">
         <v>1</v>
       </c>
+      <c r="L21" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M21" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N21" s="50">
         <v>50</v>
       </c>
+      <c r="N21" s="54">
+        <v>0.11560000000000001</v>
+      </c>
       <c r="O21" s="54">
-        <v>0.11560000000000001</v>
-      </c>
-      <c r="P21" s="54">
-        <f>O21*N21</f>
+        <f t="shared" si="0"/>
         <v>5.78</v>
       </c>
+      <c r="P21" s="52"/>
       <c r="Q21" s="52"/>
-      <c r="R21" s="52"/>
-      <c r="T21" s="77"/>
-      <c r="V21" s="77"/>
-    </row>
-    <row r="22" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S21" s="67"/>
+      <c r="U21" s="67"/>
+    </row>
+    <row r="22" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="38">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
       <c r="C22" s="59" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D22" s="46" t="s">
         <v>19</v>
@@ -2601,44 +2482,41 @@
         <v>106</v>
       </c>
       <c r="I22" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J22" s="46" t="s">
-        <v>164</v>
-      </c>
-      <c r="K22" s="46" t="s">
         <v>125</v>
       </c>
-      <c r="L22" s="47">
+      <c r="K22" s="47">
         <v>1</v>
       </c>
+      <c r="L22" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M22" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N22" s="46">
         <v>15</v>
       </c>
+      <c r="N22" s="53">
+        <v>0.19790000000000002</v>
+      </c>
       <c r="O22" s="53">
-        <v>0.19790000000000002</v>
-      </c>
-      <c r="P22" s="53">
-        <f>O22*N22</f>
+        <f t="shared" si="0"/>
         <v>2.9685000000000001</v>
       </c>
+      <c r="P22" s="48"/>
       <c r="Q22" s="48"/>
-      <c r="R22" s="48"/>
-      <c r="T22" s="77"/>
-      <c r="V22" s="77"/>
-    </row>
-    <row r="23" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S22" s="67"/>
+      <c r="U22" s="67"/>
+    </row>
+    <row r="23" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C23" s="60" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D23" s="50" t="s">
         <v>20</v>
@@ -2656,44 +2534,41 @@
         <v>107</v>
       </c>
       <c r="I23" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J23" s="50" t="s">
-        <v>165</v>
-      </c>
-      <c r="K23" s="50" t="s">
         <v>126</v>
       </c>
-      <c r="L23" s="51">
+      <c r="K23" s="51">
         <v>1</v>
       </c>
+      <c r="L23" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M23" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N23" s="50">
         <v>20</v>
       </c>
+      <c r="N23" s="54">
+        <v>0.1421</v>
+      </c>
       <c r="O23" s="54">
-        <v>0.1421</v>
-      </c>
-      <c r="P23" s="54">
-        <f>O23*N23</f>
+        <f t="shared" si="0"/>
         <v>2.8420000000000001</v>
       </c>
+      <c r="P23" s="52"/>
       <c r="Q23" s="52"/>
-      <c r="R23" s="52"/>
-      <c r="T23" s="77"/>
-      <c r="V23" s="77"/>
-    </row>
-    <row r="24" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S23" s="67"/>
+      <c r="U23" s="67"/>
+    </row>
+    <row r="24" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="38">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
       <c r="C24" s="59" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D24" s="46" t="s">
         <v>21</v>
@@ -2711,44 +2586,41 @@
         <v>108</v>
       </c>
       <c r="I24" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J24" s="46" t="s">
-        <v>166</v>
-      </c>
-      <c r="K24" s="46" t="s">
         <v>127</v>
       </c>
-      <c r="L24" s="47">
+      <c r="K24" s="47">
         <v>1</v>
       </c>
+      <c r="L24" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M24" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N24" s="46">
         <v>20</v>
       </c>
+      <c r="N24" s="53">
+        <v>0.16930000000000001</v>
+      </c>
       <c r="O24" s="53">
-        <v>0.16930000000000001</v>
-      </c>
-      <c r="P24" s="53">
-        <f>O24*N24</f>
+        <f t="shared" si="0"/>
         <v>3.3860000000000001</v>
       </c>
+      <c r="P24" s="48"/>
       <c r="Q24" s="48"/>
-      <c r="R24" s="48"/>
-      <c r="T24" s="77"/>
-      <c r="V24" s="77"/>
-    </row>
-    <row r="25" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S24" s="67"/>
+      <c r="U24" s="67"/>
+    </row>
+    <row r="25" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C25" s="60" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D25" s="50" t="s">
         <v>22</v>
@@ -2757,7 +2629,7 @@
         <v>51</v>
       </c>
       <c r="F25" s="50" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="G25" s="51" t="s">
         <v>73</v>
@@ -2766,44 +2638,41 @@
         <v>109</v>
       </c>
       <c r="I25" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J25" s="50" t="s">
-        <v>167</v>
-      </c>
-      <c r="K25" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="L25" s="51">
+        <v>159</v>
+      </c>
+      <c r="K25" s="51">
         <v>2</v>
       </c>
+      <c r="L25" s="50">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="M25" s="50">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N25" s="50">
         <v>25</v>
       </c>
+      <c r="N25" s="54">
+        <v>0.2351</v>
+      </c>
       <c r="O25" s="54">
-        <v>0.2351</v>
-      </c>
-      <c r="P25" s="54">
-        <f>O25*N25</f>
+        <f t="shared" si="0"/>
         <v>5.8775000000000004</v>
       </c>
+      <c r="P25" s="52"/>
       <c r="Q25" s="52"/>
-      <c r="R25" s="52"/>
-      <c r="T25" s="77"/>
-      <c r="V25" s="77"/>
-    </row>
-    <row r="26" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S25" s="67"/>
+      <c r="U25" s="67"/>
+    </row>
+    <row r="26" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="38">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
       <c r="C26" s="59" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D26" s="46" t="s">
         <v>23</v>
@@ -2821,44 +2690,41 @@
         <v>104</v>
       </c>
       <c r="I26" s="46" t="s">
-        <v>196</v>
+        <v>172</v>
       </c>
       <c r="J26" s="46" t="s">
-        <v>168</v>
-      </c>
-      <c r="K26" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="L26" s="47">
+        <v>159</v>
+      </c>
+      <c r="K26" s="47">
         <v>2</v>
       </c>
+      <c r="L26" s="46">
+        <f t="shared" si="2"/>
+        <v>20</v>
+      </c>
       <c r="M26" s="46">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N26" s="46">
         <v>40</v>
       </c>
+      <c r="N26" s="53">
+        <v>0.1268</v>
+      </c>
       <c r="O26" s="53">
-        <v>0.13140000000000002</v>
-      </c>
-      <c r="P26" s="53">
-        <f>O26*N26</f>
-        <v>5.2560000000000002</v>
-      </c>
+        <f t="shared" si="0"/>
+        <v>5.0720000000000001</v>
+      </c>
+      <c r="P26" s="48"/>
       <c r="Q26" s="48"/>
-      <c r="R26" s="48"/>
-      <c r="T26" s="77"/>
-      <c r="V26" s="77"/>
-    </row>
-    <row r="27" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S26" s="67"/>
+      <c r="U26" s="67"/>
+    </row>
+    <row r="27" spans="1:21" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C27" s="60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D27" s="50" t="s">
         <v>24</v>
@@ -2873,47 +2739,44 @@
         <v>128</v>
       </c>
       <c r="H27" s="50" t="s">
-        <v>194</v>
+        <v>167</v>
       </c>
       <c r="I27" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J27" s="50" t="s">
-        <v>169</v>
-      </c>
-      <c r="K27" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="L27" s="51">
+        <v>159</v>
+      </c>
+      <c r="K27" s="51">
         <v>1</v>
       </c>
+      <c r="L27" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M27" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N27" s="50">
         <v>20</v>
       </c>
+      <c r="N27" s="54">
+        <v>0.12190000000000001</v>
+      </c>
       <c r="O27" s="54">
-        <v>0.12190000000000001</v>
-      </c>
-      <c r="P27" s="54">
-        <f>O27*N27</f>
+        <f t="shared" si="0"/>
         <v>2.4380000000000002</v>
       </c>
+      <c r="P27" s="52"/>
       <c r="Q27" s="52"/>
-      <c r="R27" s="52"/>
-      <c r="T27" s="77"/>
-      <c r="V27" s="77"/>
-    </row>
-    <row r="28" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S27" s="67"/>
+      <c r="U27" s="67"/>
+    </row>
+    <row r="28" spans="1:21" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="38">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="59" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D28" s="46" t="s">
         <v>25</v>
@@ -2928,47 +2791,44 @@
         <v>129</v>
       </c>
       <c r="H28" s="46" t="s">
-        <v>193</v>
+        <v>166</v>
       </c>
       <c r="I28" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J28" s="46" t="s">
-        <v>170</v>
-      </c>
-      <c r="K28" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="L28" s="47">
+        <v>159</v>
+      </c>
+      <c r="K28" s="47">
         <v>1</v>
       </c>
+      <c r="L28" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M28" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N28" s="46">
         <v>15</v>
       </c>
+      <c r="N28" s="53">
+        <v>0.30269999999999997</v>
+      </c>
       <c r="O28" s="53">
-        <v>0.30269999999999997</v>
-      </c>
-      <c r="P28" s="53">
-        <f>O28*N28</f>
+        <f t="shared" si="0"/>
         <v>4.5404999999999998</v>
       </c>
+      <c r="P28" s="48"/>
       <c r="Q28" s="48"/>
-      <c r="R28" s="48"/>
-      <c r="T28" s="77"/>
-      <c r="V28" s="77"/>
-    </row>
-    <row r="29" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S28" s="67"/>
+      <c r="U28" s="67"/>
+    </row>
+    <row r="29" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C29" s="60" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D29" s="50" t="s">
         <v>26</v>
@@ -2980,50 +2840,47 @@
         <v>77</v>
       </c>
       <c r="G29" s="63" t="s">
-        <v>184</v>
+        <v>157</v>
       </c>
       <c r="H29" s="50" t="s">
         <v>110</v>
       </c>
       <c r="I29" s="50" t="s">
-        <v>195</v>
+        <v>168</v>
       </c>
       <c r="J29" s="50" t="s">
-        <v>171</v>
-      </c>
-      <c r="K29" s="50" t="s">
         <v>130</v>
       </c>
-      <c r="L29" s="51">
+      <c r="K29" s="51">
         <v>1</v>
       </c>
+      <c r="L29" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M29" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N29" s="50">
         <v>100</v>
       </c>
+      <c r="N29" s="54">
+        <v>0.1014</v>
+      </c>
       <c r="O29" s="54">
-        <v>0.1014</v>
-      </c>
-      <c r="P29" s="54">
-        <f>O29*N29</f>
+        <f t="shared" si="0"/>
         <v>10.14</v>
       </c>
+      <c r="P29" s="52"/>
       <c r="Q29" s="52"/>
-      <c r="R29" s="52"/>
-      <c r="T29" s="77"/>
-      <c r="V29" s="77"/>
-    </row>
-    <row r="30" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S29" s="67"/>
+      <c r="U29" s="67"/>
+    </row>
+    <row r="30" spans="1:21" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="38">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="59" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D30" s="46" t="s">
         <v>27</v>
@@ -3041,44 +2898,41 @@
         <v>100</v>
       </c>
       <c r="I30" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J30" s="46" t="s">
-        <v>172</v>
-      </c>
-      <c r="K30" s="46" t="s">
         <v>131</v>
       </c>
-      <c r="L30" s="47">
+      <c r="K30" s="47">
         <v>8</v>
       </c>
+      <c r="L30" s="46">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
       <c r="M30" s="46">
-        <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="N30" s="46">
         <v>100</v>
       </c>
+      <c r="N30" s="53">
+        <v>0.1017</v>
+      </c>
       <c r="O30" s="53">
-        <v>0.1017</v>
-      </c>
-      <c r="P30" s="53">
-        <f>O30*N30</f>
+        <f t="shared" si="0"/>
         <v>10.17</v>
       </c>
+      <c r="P30" s="48"/>
       <c r="Q30" s="48"/>
-      <c r="R30" s="48"/>
-      <c r="T30" s="77"/>
-      <c r="V30" s="77"/>
-    </row>
-    <row r="31" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S30" s="67"/>
+      <c r="U30" s="67"/>
+    </row>
+    <row r="31" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C31" s="60" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D31" s="50" t="s">
         <v>28</v>
@@ -3096,44 +2950,41 @@
         <v>111</v>
       </c>
       <c r="I31" s="50" t="s">
-        <v>197</v>
+        <v>169</v>
       </c>
       <c r="J31" s="50" t="s">
-        <v>173</v>
-      </c>
-      <c r="K31" s="50" t="s">
         <v>132</v>
       </c>
-      <c r="L31" s="51">
+      <c r="K31" s="51">
         <v>1</v>
       </c>
+      <c r="L31" s="50">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M31" s="50">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N31" s="50">
         <v>100</v>
       </c>
+      <c r="N31" s="54">
+        <v>0.10070000000000001</v>
+      </c>
       <c r="O31" s="54">
-        <v>0.10070000000000001</v>
-      </c>
-      <c r="P31" s="54">
-        <f>O31*N31</f>
+        <f t="shared" si="0"/>
         <v>10.07</v>
       </c>
+      <c r="P31" s="52"/>
       <c r="Q31" s="52"/>
-      <c r="R31" s="52"/>
-      <c r="T31" s="77"/>
-      <c r="V31" s="77"/>
-    </row>
-    <row r="32" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S31" s="67"/>
+      <c r="U31" s="67"/>
+    </row>
+    <row r="32" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="38">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
       <c r="C32" s="59" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D32" s="46" t="s">
         <v>29</v>
@@ -3151,44 +3002,41 @@
         <v>100</v>
       </c>
       <c r="I32" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J32" s="46" t="s">
-        <v>174</v>
-      </c>
-      <c r="K32" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="L32" s="47">
+      <c r="K32" s="47">
         <v>1</v>
       </c>
+      <c r="L32" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M32" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N32" s="46">
         <v>100</v>
       </c>
+      <c r="N32" s="53">
+        <v>0.10100000000000001</v>
+      </c>
       <c r="O32" s="53">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="P32" s="53">
-        <f>O32*N32</f>
+        <f t="shared" si="0"/>
         <v>10.100000000000001</v>
       </c>
+      <c r="P32" s="48"/>
       <c r="Q32" s="48"/>
-      <c r="R32" s="48"/>
-      <c r="T32" s="77"/>
-      <c r="V32" s="77"/>
-    </row>
-    <row r="33" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S32" s="67"/>
+      <c r="U32" s="67"/>
+    </row>
+    <row r="33" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C33" s="60" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D33" s="50" t="s">
         <v>30</v>
@@ -3206,37 +3054,34 @@
         <v>100</v>
       </c>
       <c r="I33" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J33" s="50" t="s">
-        <v>175</v>
-      </c>
-      <c r="K33" s="50" t="s">
         <v>134</v>
       </c>
-      <c r="L33" s="51">
+      <c r="K33" s="51">
         <v>4</v>
       </c>
+      <c r="L33" s="50">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
       <c r="M33" s="50">
-        <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-      <c r="N33" s="50">
         <v>100</v>
       </c>
+      <c r="N33" s="54">
+        <v>0.10120000000000001</v>
+      </c>
       <c r="O33" s="54">
-        <v>0.10120000000000001</v>
-      </c>
-      <c r="P33" s="54">
-        <f>O33*N33</f>
+        <f t="shared" si="0"/>
         <v>10.120000000000001</v>
       </c>
+      <c r="P33" s="52"/>
       <c r="Q33" s="52"/>
-      <c r="R33" s="52"/>
-      <c r="T33" s="77"/>
-      <c r="V33" s="77"/>
-    </row>
-    <row r="34" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S33" s="67"/>
+      <c r="U33" s="67"/>
+    </row>
+    <row r="34" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="38">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -3252,56 +3097,53 @@
         <v>60</v>
       </c>
       <c r="F34" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="G34" s="47" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="H34" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="I34" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J34" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="K34" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="L34" s="47">
+        <v>159</v>
+      </c>
+      <c r="K34" s="47">
         <v>5</v>
       </c>
-      <c r="M34" s="46">
-        <f t="shared" si="1"/>
+      <c r="L34" s="46">
+        <f t="shared" si="2"/>
         <v>50</v>
       </c>
-      <c r="N34" s="46" t="s">
-        <v>186</v>
+      <c r="M34" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="N34" s="53" t="s">
+        <v>159</v>
       </c>
       <c r="O34" s="53" t="s">
-        <v>186</v>
-      </c>
-      <c r="P34" s="53" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q34" s="62" t="s">
-        <v>187</v>
-      </c>
-      <c r="R34" s="53" t="s">
-        <v>186</v>
-      </c>
-      <c r="T34" s="77"/>
-      <c r="V34" s="77"/>
-    </row>
-    <row r="35" spans="1:22" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>159</v>
+      </c>
+      <c r="P34" s="62" t="s">
+        <v>160</v>
+      </c>
+      <c r="Q34" s="53" t="s">
+        <v>159</v>
+      </c>
+      <c r="S34" s="67"/>
+      <c r="U34" s="67"/>
+    </row>
+    <row r="35" spans="1:21" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C35" s="60" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D35" s="50" t="s">
         <v>32</v>
@@ -3310,7 +3152,7 @@
         <v>61</v>
       </c>
       <c r="F35" s="50" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="G35" s="51" t="s">
         <v>96</v>
@@ -3319,44 +3161,41 @@
         <v>112</v>
       </c>
       <c r="I35" s="50" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J35" s="50" t="s">
-        <v>176</v>
-      </c>
-      <c r="K35" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="L35" s="51">
+        <v>159</v>
+      </c>
+      <c r="K35" s="51">
         <v>3</v>
       </c>
+      <c r="L35" s="50">
+        <f t="shared" si="2"/>
+        <v>30</v>
+      </c>
       <c r="M35" s="50">
-        <f t="shared" si="1"/>
-        <v>30</v>
-      </c>
-      <c r="N35" s="50">
         <v>33</v>
       </c>
+      <c r="N35" s="54">
+        <v>0.37519999999999998</v>
+      </c>
       <c r="O35" s="54">
-        <v>0.37519999999999998</v>
-      </c>
-      <c r="P35" s="54">
-        <f>O35*N35</f>
+        <f>N35*M35</f>
         <v>12.381599999999999</v>
       </c>
+      <c r="P35" s="52"/>
       <c r="Q35" s="52"/>
-      <c r="R35" s="52"/>
-      <c r="T35" s="77"/>
-      <c r="V35" s="77"/>
-    </row>
-    <row r="36" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S35" s="67"/>
+      <c r="U35" s="67"/>
+    </row>
+    <row r="36" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="38">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="59" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D36" s="46" t="s">
         <v>33</v>
@@ -3374,44 +3213,41 @@
         <v>113</v>
       </c>
       <c r="I36" s="46" t="s">
-        <v>186</v>
+        <v>159</v>
       </c>
       <c r="J36" s="46" t="s">
-        <v>177</v>
-      </c>
-      <c r="K36" s="46" t="s">
-        <v>186</v>
-      </c>
-      <c r="L36" s="47">
+        <v>159</v>
+      </c>
+      <c r="K36" s="47">
         <v>1</v>
       </c>
+      <c r="L36" s="46">
+        <f t="shared" si="2"/>
+        <v>10</v>
+      </c>
       <c r="M36" s="46">
-        <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-      <c r="N36" s="46">
         <v>11</v>
       </c>
+      <c r="N36" s="53">
+        <v>2.5839000000000003</v>
+      </c>
       <c r="O36" s="53">
-        <v>2.5839000000000003</v>
-      </c>
-      <c r="P36" s="53">
-        <f>O36*N36</f>
+        <f>N36*M36</f>
         <v>28.422900000000002</v>
       </c>
+      <c r="P36" s="48"/>
       <c r="Q36" s="48"/>
-      <c r="R36" s="48"/>
-      <c r="T36" s="77"/>
-      <c r="V36" s="77"/>
-    </row>
-    <row r="37" spans="1:22" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S36" s="67"/>
+      <c r="U36" s="67"/>
+    </row>
+    <row r="37" spans="1:21" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="38">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="C37" s="60" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D37" s="50" t="s">
         <v>34</v>
@@ -3429,35 +3265,34 @@
         <v>114</v>
       </c>
       <c r="I37" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="J37" s="50"/>
-      <c r="K37" s="50" t="s">
-        <v>186</v>
-      </c>
-      <c r="L37" s="51">
+        <v>159</v>
+      </c>
+      <c r="J37" s="50" t="s">
+        <v>159</v>
+      </c>
+      <c r="K37" s="51">
         <v>1</v>
       </c>
-      <c r="M37" s="61">
-        <f t="shared" si="1"/>
+      <c r="L37" s="61">
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="N37" s="50">
+      <c r="M37" s="50">
         <v>11</v>
       </c>
+      <c r="N37" s="54">
+        <v>5.25</v>
+      </c>
       <c r="O37" s="54">
-        <v>5.25</v>
-      </c>
-      <c r="P37" s="54">
-        <f>O37*N37</f>
+        <f>N37*M37</f>
         <v>57.75</v>
       </c>
+      <c r="P37" s="52"/>
       <c r="Q37" s="52"/>
-      <c r="R37" s="52"/>
-      <c r="T37" s="77"/>
-      <c r="V37" s="77"/>
-    </row>
-    <row r="38" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S37" s="67"/>
+      <c r="U37" s="67"/>
+    </row>
+    <row r="38" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="33"/>
       <c r="C38" s="44"/>
@@ -3467,22 +3302,21 @@
       <c r="G38" s="37"/>
       <c r="H38" s="36"/>
       <c r="I38" s="37"/>
-      <c r="J38" s="36"/>
+      <c r="J38" s="37"/>
       <c r="K38" s="37"/>
       <c r="L38" s="37"/>
-      <c r="M38" s="37"/>
-      <c r="N38" s="75" t="s">
-        <v>198</v>
-      </c>
-      <c r="O38" s="76"/>
-      <c r="P38" s="65">
-        <f>SUM(P10:P37)</f>
-        <v>257.33039999999994</v>
-      </c>
-      <c r="Q38" s="71"/>
-      <c r="R38" s="72"/>
-    </row>
-    <row r="39" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="M38" s="76" t="s">
+        <v>170</v>
+      </c>
+      <c r="N38" s="77"/>
+      <c r="O38" s="65">
+        <f>SUM(O10:O37)</f>
+        <v>257.14639999999997</v>
+      </c>
+      <c r="P38" s="72"/>
+      <c r="Q38" s="73"/>
+    </row>
+    <row r="39" spans="1:21" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="25"/>
       <c r="C39" s="45"/>
@@ -3495,25 +3329,24 @@
       <c r="J39" s="10"/>
       <c r="K39" s="10"/>
       <c r="L39" s="10"/>
-      <c r="M39" s="10"/>
-      <c r="N39" s="75" t="s">
-        <v>199</v>
-      </c>
-      <c r="O39" s="76"/>
-      <c r="P39" s="66">
-        <f>P38/10</f>
-        <v>25.733039999999995</v>
-      </c>
-      <c r="Q39" s="73"/>
-      <c r="R39" s="74"/>
+      <c r="M39" s="76" t="s">
+        <v>171</v>
+      </c>
+      <c r="N39" s="77"/>
+      <c r="O39" s="66">
+        <f>O38/10</f>
+        <v>25.714639999999996</v>
+      </c>
+      <c r="P39" s="74"/>
+      <c r="Q39" s="75"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="K1:R1"/>
-    <mergeCell ref="R3:R8"/>
-    <mergeCell ref="Q38:R39"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="J1:Q1"/>
+    <mergeCell ref="Q3:Q8"/>
+    <mergeCell ref="P38:Q39"/>
+    <mergeCell ref="M38:N38"/>
+    <mergeCell ref="M39:N39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>